<commit_message>
Update scale plan, segment map, and add reference files
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scale/segment-map.xlsx
+++ b/scale/segment-map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20367"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\scripts\scale\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{36F94BAA-609C-4ACB-8A95-11BC391742AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB588ABE-F2B7-4F82-A850-E3DC34F139EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5196CB33-50D7-47E6-A36A-3F222C6487A7}"/>
   </bookViews>
@@ -118,7 +118,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -435,7 +435,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -550,6 +550,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -595,12 +610,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -979,257 +997,258 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C71FF281-4C2A-45AD-8B15-05D4BCA81CCD}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.3984375" style="1" customWidth="1"/>
     <col min="2" max="2" width="17" style="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.3984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.19921875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.796875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+    <row r="2" spans="1:6">
+      <c r="A2" s="3">
         <v>46085</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>57000</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <v>39000</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+    <row r="3" spans="1:6">
+      <c r="A3" s="3">
         <v>46085</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>7</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>79000</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>54000</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+    <row r="4" spans="1:6">
+      <c r="A4" s="3">
         <v>46085</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>7</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>10000</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="2">
         <v>7300</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+    <row r="5" spans="1:6">
+      <c r="A5" s="3">
         <v>46085</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>3</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>12000</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <v>7000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+    <row r="6" spans="1:6">
+      <c r="A6" s="3">
         <v>46085</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>11</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>16000</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <v>7700</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+    <row r="7" spans="1:6">
+      <c r="A7" s="3">
         <v>46085</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+    <row r="8" spans="1:6">
+      <c r="A8" s="3">
         <v>46085</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>16000</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="2">
         <v>7900</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+    <row r="9" spans="1:6">
+      <c r="A9" s="3">
         <v>46085</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="2">
         <v>8</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>21000</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="2">
         <v>9400</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+    <row r="10" spans="1:6">
+      <c r="A10" s="3">
         <v>46085</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="2">
         <v>10</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>18000</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="2">
         <v>8700</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+    <row r="11" spans="1:6">
+      <c r="A11" s="3">
         <v>46085</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="2">
         <v>10</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>8000</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="2">
         <v>3600</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
+    <row r="12" spans="1:6">
+      <c r="A12" s="3">
         <v>46085</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>7</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>12000</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="2">
         <v>5900</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add meeting rules, update segment map, remove completed pricing review
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scale/segment-map.xlsx
+++ b/scale/segment-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20367"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\scripts\scale\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB588ABE-F2B7-4F82-A850-E3DC34F139EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388CA578-C8AE-45BD-8E10-A38DB19BC45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5196CB33-50D7-47E6-A36A-3F222C6487A7}"/>
+    <workbookView xWindow="11232" yWindow="1440" windowWidth="11808" windowHeight="10800" xr2:uid="{5196CB33-50D7-47E6-A36A-3F222C6487A7}"/>
   </bookViews>
   <sheets>
     <sheet name="segment-map" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>IVES-WHITE</t>
   </si>
@@ -112,13 +112,19 @@
   </si>
   <si>
     <t>GP</t>
+  </si>
+  <si>
+    <t>MAYARI</t>
+  </si>
+  <si>
+    <t>Mayari</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -996,18 +1002,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C71FF281-4C2A-45AD-8B15-05D4BCA81CCD}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.3984375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="17" style="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.3984375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.19921875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -1027,7 +1033,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>46085</v>
       </c>
@@ -1047,7 +1053,7 @@
         <v>39000</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>46085</v>
       </c>
@@ -1067,7 +1073,7 @@
         <v>54000</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>46085</v>
       </c>
@@ -1087,7 +1093,7 @@
         <v>7300</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>46085</v>
       </c>
@@ -1107,7 +1113,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>46085</v>
       </c>
@@ -1127,7 +1133,7 @@
         <v>7700</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>46085</v>
       </c>
@@ -1147,7 +1153,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>46085</v>
       </c>
@@ -1167,7 +1173,7 @@
         <v>7900</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>46085</v>
       </c>
@@ -1187,7 +1193,7 @@
         <v>9400</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>46085</v>
       </c>
@@ -1207,7 +1213,7 @@
         <v>8700</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>46085</v>
       </c>
@@ -1227,7 +1233,7 @@
         <v>3600</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>46085</v>
       </c>
@@ -1245,6 +1251,26 @@
       </c>
       <c r="F12" s="2">
         <v>5900</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>46085</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="2">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2">
+        <v>7000</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>